<commit_message>
chore(e2e): ship the CSV and XLSX import samples alongside the fixture
Only bookings-valid.xlsx was ever committed; the CSV counterparts existed
outside the repo, so there was nothing on the branch to drag into the import
dialog by hand. All five now live in e2e/fixtures.

Regenerated against the current schema: every file gains a payments column,
one row carries a real payment schedule (paid + unpaid, summing with the
deposit to exactly the total), and errors.csv swaps its malformed-booking_id
row for a malformed-payments one — a non-ObjectId booking_id is a grouping key
now, not an error.

Row counts are unchanged, so the XLSX preview assertion still reads 6 of 6.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012A3Yvy1qbGbyVsVLRAKvj9
</commit_message>
<xml_diff>
--- a/e2e/fixtures/bookings-valid.xlsx
+++ b/e2e/fixtures/bookings-valid.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="71">
   <si>
     <t>clientName</t>
   </si>
@@ -67,6 +67,9 @@
     <t>locationLng</t>
   </si>
   <si>
+    <t>payments</t>
+  </si>
+  <si>
     <t>Marisol Reyes</t>
   </si>
   <si>
@@ -113,6 +116,9 @@
   </si>
   <si>
     <t>120.9621</t>
+  </si>
+  <si>
+    <t>[{"price":40000,"status":"paid","title":"Second instalment","method":"remit","paidAt":"2026-07-01T00:00:00.000Z"},{"price":90000,"status":"unpaid","title":"Balance on the day","method":"cash"}]</t>
   </si>
   <si>
     <t>Diego Alonzo</t>
@@ -594,10 +600,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -652,341 +658,362 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" t="s">
         <v>25</v>
       </c>
-      <c r="I2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="H3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" t="s">
         <v>28</v>
       </c>
-      <c r="L2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" t="s">
-        <v>30</v>
-      </c>
-      <c r="N2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" t="s">
-        <v>30</v>
-      </c>
-      <c r="P2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" t="s">
-        <v>33</v>
+      <c r="K3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" t="s">
+        <v>46</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R3" t="s">
+        <v>31</v>
+      </c>
+      <c r="S3" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>36</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B4" t="s">
         <v>37</v>
       </c>
-      <c r="E3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" t="s">
         <v>40</v>
       </c>
-      <c r="I3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J3" t="s">
-        <v>27</v>
-      </c>
-      <c r="K3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L3" t="s">
-        <v>30</v>
-      </c>
-      <c r="M3" t="s">
-        <v>43</v>
-      </c>
-      <c r="N3" t="s">
-        <v>44</v>
-      </c>
-      <c r="O3" t="s">
-        <v>30</v>
-      </c>
-      <c r="P3" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>30</v>
-      </c>
-      <c r="R3" t="s">
-        <v>30</v>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" t="s">
+        <v>31</v>
+      </c>
+      <c r="M4" t="s">
+        <v>45</v>
+      </c>
+      <c r="N4" t="s">
+        <v>49</v>
+      </c>
+      <c r="O4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R4" t="s">
+        <v>31</v>
+      </c>
+      <c r="S4" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" t="s">
-        <v>30</v>
-      </c>
-      <c r="L4" t="s">
-        <v>30</v>
-      </c>
-      <c r="M4" t="s">
-        <v>43</v>
-      </c>
-      <c r="N4" t="s">
-        <v>47</v>
-      </c>
-      <c r="O4" t="s">
-        <v>30</v>
-      </c>
-      <c r="P4" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>30</v>
-      </c>
-      <c r="R4" t="s">
-        <v>30</v>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" t="s">
+        <v>31</v>
+      </c>
+      <c r="L5" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>31</v>
+      </c>
+      <c r="R5" t="s">
+        <v>31</v>
+      </c>
+      <c r="S5" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" t="s">
-        <v>30</v>
-      </c>
-      <c r="L5" t="s">
-        <v>54</v>
-      </c>
-      <c r="M5" t="s">
-        <v>30</v>
-      </c>
-      <c r="N5" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" t="s">
-        <v>30</v>
-      </c>
-      <c r="P5" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>30</v>
-      </c>
-      <c r="R5" t="s">
-        <v>30</v>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" t="s">
+        <v>66</v>
+      </c>
+      <c r="L6" t="s">
+        <v>67</v>
+      </c>
+      <c r="M6" t="s">
+        <v>31</v>
+      </c>
+      <c r="N6" t="s">
+        <v>31</v>
+      </c>
+      <c r="O6" t="s">
+        <v>31</v>
+      </c>
+      <c r="P6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6" t="s">
+        <v>31</v>
+      </c>
+      <c r="S6" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" t="s">
-        <v>62</v>
-      </c>
-      <c r="I6" t="s">
-        <v>63</v>
-      </c>
-      <c r="J6" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" t="s">
-        <v>64</v>
-      </c>
-      <c r="L6" t="s">
-        <v>65</v>
-      </c>
-      <c r="M6" t="s">
-        <v>30</v>
-      </c>
-      <c r="N6" t="s">
-        <v>30</v>
-      </c>
-      <c r="O6" t="s">
-        <v>30</v>
-      </c>
-      <c r="P6" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>30</v>
-      </c>
-      <c r="R6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R7" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="S7" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>